<commit_message>
TMTI0045472- Feb 23 2024 , Browser Zoom In
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeRecordManagerForFVACAOUserOntheSFLightningView.xlsx
+++ b/TestData/LV_TMTT0038660_VerifyTheFunctionalityOfTimeRecordManagerForFVACAOUserOntheSFLightningView.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{343A6B25-A859-4940-83EF-429852311BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4FEE9C-95E2-4238-A968-7A2F15359716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
     <sheet name="AppName" sheetId="12" r:id="rId2"/>
     <sheet name="ModuleName" sheetId="13" r:id="rId3"/>
-    <sheet name="SummaryLogs" sheetId="7" r:id="rId4"/>
-    <sheet name="DetailLogs" sheetId="11" r:id="rId5"/>
-    <sheet name="RateSheetManagement" sheetId="9" r:id="rId6"/>
-    <sheet name="StaffMember" sheetId="10" r:id="rId7"/>
-    <sheet name="UpdateData" sheetId="14" r:id="rId8"/>
+    <sheet name="WeeklyEntryMatrix" sheetId="15" r:id="rId4"/>
+    <sheet name="SummaryLogs" sheetId="7" r:id="rId5"/>
+    <sheet name="DetailLogs" sheetId="11" r:id="rId6"/>
+    <sheet name="RateSheetManagement" sheetId="9" r:id="rId7"/>
+    <sheet name="StaffMember" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="49">
   <si>
     <t>Global Search User</t>
   </si>
@@ -108,12 +108,6 @@
     <t>8</t>
   </si>
   <si>
-    <t>Conduct Research</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>GroupName</t>
   </si>
   <si>
@@ -144,9 +138,6 @@
     <t>Project Omaha - FDD-Congruex-FVA-106209</t>
   </si>
   <si>
-    <t>Project Omaha - FDD - 106209</t>
-  </si>
-  <si>
     <t>Time Tracking Beta Supervisor</t>
   </si>
   <si>
@@ -154,6 +145,51 @@
   </si>
   <si>
     <t>T</t>
+  </si>
+  <si>
+    <t>Sasha Johnson</t>
+  </si>
+  <si>
+    <t>Christy Skaar</t>
+  </si>
+  <si>
+    <t>Akshay Joshi</t>
+  </si>
+  <si>
+    <t>Palladium - Q1 2016-Palladium Equity Partners-FVA-24718</t>
+  </si>
+  <si>
+    <t>Closing/Bring Down</t>
+  </si>
+  <si>
+    <t>Palladium - Q1 2016 - FVA - 24718</t>
+  </si>
+  <si>
+    <t>Blaise Brunda</t>
+  </si>
+  <si>
+    <t>Apeksha Saini</t>
+  </si>
+  <si>
+    <t>Director Rate</t>
+  </si>
+  <si>
+    <t>Project Blue Bird-bluebird bio, Inc.-FVA-122491</t>
+  </si>
+  <si>
+    <t>Project Blue Bird - FVA - 122491</t>
+  </si>
+  <si>
+    <t>Time Tracking TFR Supervisor</t>
+  </si>
+  <si>
+    <t>Time Tracking PV Supervisor</t>
+  </si>
+  <si>
+    <t>Project Beach-StoicLane-FVA-121929</t>
+  </si>
+  <si>
+    <t>Project Beach - FVA - 121929</t>
   </si>
 </sst>
 </file>
@@ -192,7 +228,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -200,16 +236,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -498,26 +550,29 @@
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
         <v>23</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -570,14 +625,92 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7F57535-9BF1-4641-B5A5-76DE623B9558}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="53.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -587,7 +720,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -604,13 +737,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -620,6 +753,28 @@
       </c>
       <c r="F2" s="2" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -628,9 +783,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" bestFit="1" customWidth="1"/>
@@ -663,13 +818,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>11</v>
@@ -679,6 +834,28 @@
       </c>
       <c r="F2" s="2" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -687,12 +864,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="53.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="61.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -705,18 +882,40 @@
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>33</v>
       </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>36</v>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -725,13 +924,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -747,24 +946,36 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+      <c r="A3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
+      <c r="A4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
@@ -773,35 +984,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C72E838B-CDBC-4DB0-BF1D-AC44E1CE047A}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>